<commit_message>
fix assay scaffold writing
</commit_message>
<xml_diff>
--- a/tests/ProcessCore.Tests/TestObjects/fct_gcqtof_assay.xlsx
+++ b/tests/ProcessCore.Tests/TestObjects/fct_gcqtof_assay.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F99EDA-FA90-42A1-BAD9-08813BA15E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2652BBC-1218-49F3-80A0-C959B1DB5160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25510" yWindow="0" windowWidth="25780" windowHeight="20970" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="isa_assay" sheetId="1" r:id="rId1"/>
@@ -853,7 +853,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -992,6 +992,10 @@
     <filterColumn colId="32" hiddenButton="1"/>
     <filterColumn colId="33" hiddenButton="1"/>
   </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AH21">
+    <sortCondition ref="F2:F21"/>
+    <sortCondition descending="1" ref="AB2:AB21"/>
+  </sortState>
   <tableColumns count="34">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Input [Sample Name]" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Protocol REF"/>
@@ -1406,14 +1410,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1421,7 +1425,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1429,7 +1433,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1437,7 +1441,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -1445,17 +1449,17 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1463,7 +1467,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1471,7 +1475,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1479,7 +1483,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1487,7 +1491,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -1495,12 +1499,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1520,7 +1524,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1540,12 +1544,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -1556,7 +1560,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -1564,12 +1568,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>40</v>
       </c>
@@ -1580,7 +1584,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -1591,7 +1595,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>45</v>
       </c>
@@ -1602,7 +1606,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>47</v>
       </c>
@@ -1613,7 +1617,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>49</v>
       </c>
@@ -1624,12 +1628,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>52</v>
       </c>
@@ -1649,9 +1653,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AL7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>55</v>
       </c>
@@ -1767,7 +1771,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>93</v>
       </c>
@@ -1865,7 +1869,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>118</v>
       </c>
@@ -1963,7 +1967,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>122</v>
       </c>
@@ -2061,7 +2065,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>126</v>
       </c>
@@ -2159,7 +2163,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>130</v>
       </c>
@@ -2257,7 +2261,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>133</v>
       </c>
@@ -2367,9 +2371,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AH21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>55</v>
       </c>
@@ -2473,7 +2477,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>163</v>
       </c>
@@ -2559,9 +2563,9 @@
         <v>176</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="B3" t="s">
         <v>164</v>
@@ -2630,13 +2634,10 @@
         <v>113</v>
       </c>
       <c r="AB3" t="s">
-        <v>177</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="AD3" t="s">
-        <v>179</v>
+        <v>99</v>
       </c>
       <c r="AE3" t="s">
         <v>175</v>
@@ -2645,12 +2646,12 @@
         <v>99</v>
       </c>
       <c r="AH3" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="B4" t="s">
         <v>164</v>
@@ -2731,12 +2732,12 @@
         <v>99</v>
       </c>
       <c r="AH4" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="B5" t="s">
         <v>164</v>
@@ -2805,13 +2806,10 @@
         <v>113</v>
       </c>
       <c r="AB5" t="s">
-        <v>177</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="AD5" t="s">
-        <v>179</v>
+        <v>99</v>
       </c>
       <c r="AE5" t="s">
         <v>175</v>
@@ -2820,12 +2818,12 @@
         <v>99</v>
       </c>
       <c r="AH5" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>163</v>
       </c>
       <c r="B6" t="s">
         <v>164</v>
@@ -2840,13 +2838,13 @@
         <v>166</v>
       </c>
       <c r="F6" t="s">
-        <v>184</v>
+        <v>99</v>
       </c>
       <c r="G6" t="s">
-        <v>185</v>
+        <v>99</v>
       </c>
       <c r="H6" t="s">
-        <v>186</v>
+        <v>99</v>
       </c>
       <c r="I6" t="s">
         <v>167</v>
@@ -2894,10 +2892,13 @@
         <v>113</v>
       </c>
       <c r="AB6" t="s">
-        <v>174</v>
+        <v>177</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>178</v>
       </c>
       <c r="AD6" t="s">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="AE6" t="s">
         <v>175</v>
@@ -2906,12 +2907,12 @@
         <v>99</v>
       </c>
       <c r="AH6" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>117</v>
+        <v>181</v>
       </c>
       <c r="B7" t="s">
         <v>164</v>
@@ -2926,13 +2927,13 @@
         <v>166</v>
       </c>
       <c r="F7" t="s">
-        <v>184</v>
+        <v>99</v>
       </c>
       <c r="G7" t="s">
-        <v>185</v>
+        <v>99</v>
       </c>
       <c r="H7" t="s">
-        <v>186</v>
+        <v>99</v>
       </c>
       <c r="I7" t="s">
         <v>167</v>
@@ -2995,12 +2996,12 @@
         <v>99</v>
       </c>
       <c r="AH7" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="8" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>121</v>
+        <v>163</v>
       </c>
       <c r="B8" t="s">
         <v>164</v>
@@ -3015,13 +3016,13 @@
         <v>166</v>
       </c>
       <c r="F8" t="s">
-        <v>184</v>
+        <v>99</v>
       </c>
       <c r="G8" t="s">
-        <v>185</v>
+        <v>99</v>
       </c>
       <c r="H8" t="s">
-        <v>186</v>
+        <v>99</v>
       </c>
       <c r="I8" t="s">
         <v>167</v>
@@ -3069,10 +3070,13 @@
         <v>113</v>
       </c>
       <c r="AB8" t="s">
-        <v>174</v>
+        <v>177</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>178</v>
       </c>
       <c r="AD8" t="s">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="AE8" t="s">
         <v>175</v>
@@ -3081,12 +3085,12 @@
         <v>99</v>
       </c>
       <c r="AH8" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="9" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>121</v>
+        <v>201</v>
       </c>
       <c r="B9" t="s">
         <v>164</v>
@@ -3101,13 +3105,13 @@
         <v>166</v>
       </c>
       <c r="F9" t="s">
-        <v>184</v>
+        <v>99</v>
       </c>
       <c r="G9" t="s">
-        <v>185</v>
+        <v>99</v>
       </c>
       <c r="H9" t="s">
-        <v>186</v>
+        <v>99</v>
       </c>
       <c r="I9" t="s">
         <v>167</v>
@@ -3170,12 +3174,12 @@
         <v>99</v>
       </c>
       <c r="AH9" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="10" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="B10" t="s">
         <v>164</v>
@@ -3256,12 +3260,12 @@
         <v>99</v>
       </c>
       <c r="AH10" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="11" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B11" t="s">
         <v>164</v>
@@ -3330,13 +3334,10 @@
         <v>113</v>
       </c>
       <c r="AB11" t="s">
-        <v>177</v>
-      </c>
-      <c r="AC11" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="AD11" t="s">
-        <v>179</v>
+        <v>99</v>
       </c>
       <c r="AE11" t="s">
         <v>175</v>
@@ -3345,12 +3346,12 @@
         <v>99</v>
       </c>
       <c r="AH11" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>163</v>
+        <v>125</v>
       </c>
       <c r="B12" t="s">
         <v>164</v>
@@ -3365,13 +3366,13 @@
         <v>166</v>
       </c>
       <c r="F12" t="s">
-        <v>99</v>
+        <v>184</v>
       </c>
       <c r="G12" t="s">
-        <v>99</v>
+        <v>185</v>
       </c>
       <c r="H12" t="s">
-        <v>99</v>
+        <v>186</v>
       </c>
       <c r="I12" t="s">
         <v>167</v>
@@ -3431,12 +3432,12 @@
         <v>99</v>
       </c>
       <c r="AH12" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>163</v>
+        <v>129</v>
       </c>
       <c r="B13" t="s">
         <v>164</v>
@@ -3451,13 +3452,13 @@
         <v>166</v>
       </c>
       <c r="F13" t="s">
-        <v>99</v>
+        <v>184</v>
       </c>
       <c r="G13" t="s">
-        <v>99</v>
+        <v>185</v>
       </c>
       <c r="H13" t="s">
-        <v>99</v>
+        <v>186</v>
       </c>
       <c r="I13" t="s">
         <v>167</v>
@@ -3505,13 +3506,10 @@
         <v>113</v>
       </c>
       <c r="AB13" t="s">
-        <v>177</v>
-      </c>
-      <c r="AC13" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="AD13" t="s">
-        <v>179</v>
+        <v>99</v>
       </c>
       <c r="AE13" t="s">
         <v>175</v>
@@ -3520,12 +3518,12 @@
         <v>99</v>
       </c>
       <c r="AH13" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B14" t="s">
         <v>164</v>
@@ -3606,12 +3604,12 @@
         <v>99</v>
       </c>
       <c r="AH14" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="15" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B15" t="s">
         <v>164</v>
@@ -3680,13 +3678,10 @@
         <v>113</v>
       </c>
       <c r="AB15" t="s">
-        <v>177</v>
-      </c>
-      <c r="AC15" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="AD15" t="s">
-        <v>179</v>
+        <v>99</v>
       </c>
       <c r="AE15" t="s">
         <v>175</v>
@@ -3695,12 +3690,12 @@
         <v>99</v>
       </c>
       <c r="AH15" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="16" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="B16" t="s">
         <v>164</v>
@@ -3769,10 +3764,13 @@
         <v>113</v>
       </c>
       <c r="AB16" t="s">
-        <v>174</v>
+        <v>177</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>178</v>
       </c>
       <c r="AD16" t="s">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="AE16" t="s">
         <v>175</v>
@@ -3781,12 +3779,12 @@
         <v>99</v>
       </c>
       <c r="AH16" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="17" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="B17" t="s">
         <v>164</v>
@@ -3870,12 +3868,12 @@
         <v>99</v>
       </c>
       <c r="AH17" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="18" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="B18" t="s">
         <v>164</v>
@@ -3944,10 +3942,13 @@
         <v>113</v>
       </c>
       <c r="AB18" t="s">
-        <v>174</v>
+        <v>177</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>178</v>
       </c>
       <c r="AD18" t="s">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="AE18" t="s">
         <v>175</v>
@@ -3956,12 +3957,12 @@
         <v>99</v>
       </c>
       <c r="AH18" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="19" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B19" t="s">
         <v>164</v>
@@ -4045,12 +4046,12 @@
         <v>99</v>
       </c>
       <c r="AH19" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="20" spans="1:34" x14ac:dyDescent="0.25">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="20" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>201</v>
+        <v>132</v>
       </c>
       <c r="B20" t="s">
         <v>164</v>
@@ -4065,13 +4066,13 @@
         <v>166</v>
       </c>
       <c r="F20" t="s">
-        <v>99</v>
+        <v>184</v>
       </c>
       <c r="G20" t="s">
-        <v>99</v>
+        <v>185</v>
       </c>
       <c r="H20" t="s">
-        <v>99</v>
+        <v>186</v>
       </c>
       <c r="I20" t="s">
         <v>167</v>
@@ -4119,10 +4120,13 @@
         <v>113</v>
       </c>
       <c r="AB20" t="s">
-        <v>174</v>
+        <v>177</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>178</v>
       </c>
       <c r="AD20" t="s">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="AE20" t="s">
         <v>175</v>
@@ -4131,12 +4135,12 @@
         <v>99</v>
       </c>
       <c r="AH20" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="21" spans="1:34" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="21" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>201</v>
+        <v>135</v>
       </c>
       <c r="B21" t="s">
         <v>164</v>
@@ -4151,13 +4155,13 @@
         <v>166</v>
       </c>
       <c r="F21" t="s">
-        <v>99</v>
+        <v>184</v>
       </c>
       <c r="G21" t="s">
-        <v>99</v>
+        <v>185</v>
       </c>
       <c r="H21" t="s">
-        <v>99</v>
+        <v>186</v>
       </c>
       <c r="I21" t="s">
         <v>167</v>
@@ -4220,7 +4224,7 @@
         <v>99</v>
       </c>
       <c r="AH21" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -4235,9 +4239,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AG21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>55</v>
       </c>
@@ -4338,7 +4342,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>176</v>
       </c>
@@ -4427,7 +4431,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>180</v>
       </c>
@@ -4516,7 +4520,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>182</v>
       </c>
@@ -4605,7 +4609,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>183</v>
       </c>
@@ -4694,7 +4698,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>187</v>
       </c>
@@ -4783,7 +4787,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>188</v>
       </c>
@@ -4872,7 +4876,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>189</v>
       </c>
@@ -4961,7 +4965,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>190</v>
       </c>
@@ -5050,7 +5054,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>191</v>
       </c>
@@ -5139,7 +5143,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>192</v>
       </c>
@@ -5228,7 +5232,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>193</v>
       </c>
@@ -5317,7 +5321,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>194</v>
       </c>
@@ -5406,7 +5410,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>195</v>
       </c>
@@ -5495,7 +5499,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>196</v>
       </c>
@@ -5584,7 +5588,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>197</v>
       </c>
@@ -5673,7 +5677,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>198</v>
       </c>
@@ -5762,7 +5766,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>199</v>
       </c>
@@ -5851,7 +5855,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>200</v>
       </c>
@@ -5940,7 +5944,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>202</v>
       </c>
@@ -6029,7 +6033,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>203</v>
       </c>

</xml_diff>